<commit_message>
added feilds in csv
</commit_message>
<xml_diff>
--- a/frontend/dist/sample-result-template.xlsx
+++ b/frontend/dist/sample-result-template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jashu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0B89CDA-853E-450F-8517-1B14FEC5B404}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FC6D49D-9C75-41EA-AEC6-63526A3F0C61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D305303B-9F6A-495F-A733-32E7B5D9BF48}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
   <si>
     <t>S. No.</t>
   </si>
@@ -228,9 +228,6 @@
     <t>Academic Year</t>
   </si>
   <si>
-    <t>Course Name</t>
-  </si>
-  <si>
     <t>Exam Flag</t>
   </si>
   <si>
@@ -238,16 +235,22 @@
   </si>
   <si>
     <t>Semester</t>
+  </si>
+  <si>
+    <t>Paper Name (Hindi)</t>
+  </si>
+  <si>
+    <t>Paper Name (English)</t>
+  </si>
+  <si>
+    <t>FIELD35</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="[$-4000439]0"/>
-  </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -277,13 +280,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -305,7 +301,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -316,18 +312,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFC00000"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -341,9 +356,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -381,7 +396,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -487,7 +502,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -629,7 +644,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -637,30 +652,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E0D9494-A35D-4243-9185-AFCA14D87385}">
-  <dimension ref="A1:AH29"/>
+  <dimension ref="A1:AI2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.36328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.36328125" style="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.36328125" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.81640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.26953125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.08984375" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.08984375" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.08984375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.90625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="37.08984375" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.08984375" style="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.54296875" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="22.26953125" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="19.08984375" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.26953125" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="32.6328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="26.6328125" style="3" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="14.36328125" style="3" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="15.81640625" style="3" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="14.36328125" style="3" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="15.81640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.90625" style="3" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="11.81640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.453125" style="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.453125" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="15" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.08984375" style="3" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="16.453125" style="3" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="17.54296875" style="3" bestFit="1" customWidth="1"/>
     <col min="24" max="25" width="19" style="3" bestFit="1" customWidth="1"/>
@@ -669,13 +684,13 @@
     <col min="28" max="28" width="20.1796875" style="3" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="11.7265625" style="3" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="13.08984375" style="3" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="15.7265625" style="3" customWidth="1"/>
-    <col min="32" max="32" width="9.08984375" style="3" bestFit="1" customWidth="1"/>
-    <col min="33" max="16384" width="8.7265625" style="3"/>
+    <col min="31" max="32" width="15.7265625" style="3" customWidth="1"/>
+    <col min="33" max="33" width="9.08984375" style="3" bestFit="1" customWidth="1"/>
+    <col min="34" max="16384" width="8.7265625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:35" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="7" t="s">
         <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -693,7 +708,7 @@
       <c r="F1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="4" t="s">
         <v>10</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -777,9 +792,12 @@
       <c r="AH1" s="1" t="s">
         <v>61</v>
       </c>
+      <c r="AI1" s="1" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="2" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:35" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -792,12 +810,12 @@
         <v>2</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>32</v>
+        <v>67</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="G2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>36</v>
       </c>
       <c r="H2" s="2" t="s">
@@ -870,155 +888,26 @@
         <v>63</v>
       </c>
       <c r="AE2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="AF2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="AG2" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="AF2" s="2" t="s">
+      <c r="AH2" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="AG2" s="2" t="s">
+      <c r="AI2" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="AH2" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="B3" s="4"/>
-      <c r="G3" s="5"/>
-      <c r="AE3" s="6"/>
-    </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="B4" s="4"/>
-      <c r="G4" s="5"/>
-      <c r="AE4" s="6"/>
-    </row>
-    <row r="5" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="B5" s="4"/>
-      <c r="G5" s="5"/>
-      <c r="AE5" s="6"/>
-    </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="B6" s="4"/>
-      <c r="G6" s="5"/>
-      <c r="AE6" s="6"/>
-    </row>
-    <row r="7" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="B7" s="4"/>
-      <c r="G7" s="5"/>
-      <c r="AE7" s="6"/>
-    </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="B8" s="4"/>
-      <c r="G8" s="5"/>
-      <c r="AE8" s="6"/>
-    </row>
-    <row r="9" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="B9" s="4"/>
-      <c r="G9" s="5"/>
-      <c r="AE9" s="6"/>
-    </row>
-    <row r="10" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="B10" s="4"/>
-      <c r="G10" s="5"/>
-      <c r="AE10" s="6"/>
-    </row>
-    <row r="11" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="B11" s="4"/>
-      <c r="G11" s="5"/>
-      <c r="AE11" s="6"/>
-    </row>
-    <row r="12" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="B12" s="4"/>
-      <c r="G12" s="5"/>
-      <c r="AE12" s="6"/>
-    </row>
-    <row r="13" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="B13" s="4"/>
-      <c r="G13" s="5"/>
-      <c r="AE13" s="6"/>
-    </row>
-    <row r="14" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="B14" s="4"/>
-      <c r="G14" s="5"/>
-      <c r="AE14" s="6"/>
-    </row>
-    <row r="15" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="B15" s="4"/>
-      <c r="G15" s="5"/>
-      <c r="AE15" s="6"/>
-    </row>
-    <row r="16" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="B16" s="4"/>
-      <c r="G16" s="5"/>
-      <c r="AE16" s="6"/>
-    </row>
-    <row r="17" spans="2:31" x14ac:dyDescent="0.35">
-      <c r="B17" s="4"/>
-      <c r="G17" s="5"/>
-      <c r="AE17" s="6"/>
-    </row>
-    <row r="18" spans="2:31" x14ac:dyDescent="0.35">
-      <c r="B18" s="4"/>
-      <c r="G18" s="5"/>
-      <c r="AE18" s="6"/>
-    </row>
-    <row r="19" spans="2:31" x14ac:dyDescent="0.35">
-      <c r="B19" s="4"/>
-      <c r="G19" s="5"/>
-      <c r="AE19" s="6"/>
-    </row>
-    <row r="20" spans="2:31" x14ac:dyDescent="0.35">
-      <c r="B20" s="4"/>
-      <c r="G20" s="5"/>
-      <c r="AE20" s="6"/>
-    </row>
-    <row r="21" spans="2:31" x14ac:dyDescent="0.35">
-      <c r="B21" s="4"/>
-      <c r="G21" s="5"/>
-      <c r="AE21" s="6"/>
-    </row>
-    <row r="22" spans="2:31" x14ac:dyDescent="0.35">
-      <c r="B22" s="4"/>
-      <c r="G22" s="5"/>
-      <c r="AE22" s="6"/>
-    </row>
-    <row r="23" spans="2:31" x14ac:dyDescent="0.35">
-      <c r="B23" s="4"/>
-      <c r="G23" s="5"/>
-      <c r="AE23" s="6"/>
-    </row>
-    <row r="24" spans="2:31" x14ac:dyDescent="0.35">
-      <c r="B24" s="4"/>
-      <c r="G24" s="5"/>
-      <c r="AE24" s="6"/>
-    </row>
-    <row r="25" spans="2:31" x14ac:dyDescent="0.35">
-      <c r="B25" s="4"/>
-      <c r="G25" s="5"/>
-      <c r="AE25" s="6"/>
-    </row>
-    <row r="26" spans="2:31" x14ac:dyDescent="0.35">
-      <c r="B26" s="4"/>
-      <c r="G26" s="5"/>
-      <c r="AE26" s="6"/>
-    </row>
-    <row r="27" spans="2:31" x14ac:dyDescent="0.35">
-      <c r="B27" s="4"/>
-      <c r="G27" s="5"/>
-      <c r="AE27" s="6"/>
-    </row>
-    <row r="28" spans="2:31" x14ac:dyDescent="0.35">
-      <c r="B28" s="4"/>
-      <c r="G28" s="5"/>
-      <c r="AE28" s="6"/>
-    </row>
-    <row r="29" spans="2:31" x14ac:dyDescent="0.35">
-      <c r="B29" s="4"/>
-      <c r="G29" s="5"/>
-      <c r="AE29" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>